<commit_message>
Update Adventure Works-Clean data.xlsx
</commit_message>
<xml_diff>
--- a/Adventure Works-Clean data.xlsx
+++ b/Adventure Works-Clean data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Documents\GitHub\Excel-Adventure-Works-Dashboards\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C13156CD-9CC6-4441-A9D7-5110974DDD6E}" xr6:coauthVersionLast="41" xr6:coauthVersionMax="41" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44245BCD-153A-426B-A198-2D30DA5D2FFD}" xr6:coauthVersionLast="41" xr6:coauthVersionMax="41" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4470" yWindow="3015" windowWidth="15375" windowHeight="7785" firstSheet="1" activeTab="1" xr2:uid="{8C91DA6D-E5A1-4120-A228-5D2A48CFAB22}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="1" activeTab="1" xr2:uid="{8C91DA6D-E5A1-4120-A228-5D2A48CFAB22}"/>
   </bookViews>
   <sheets>
     <sheet name="DimCustomer" sheetId="7" r:id="rId1"/>
@@ -1333,7 +1333,7 @@
           <a:avLst/>
         </a:prstGeom>
         <a:solidFill>
-          <a:schemeClr val="tx1"/>
+          <a:schemeClr val="bg1"/>
         </a:solidFill>
         <a:ln>
           <a:noFill/>
@@ -1399,7 +1399,7 @@
           <a:avLst/>
         </a:prstGeom>
         <a:solidFill>
-          <a:schemeClr val="tx1"/>
+          <a:schemeClr val="bg1"/>
         </a:solidFill>
         <a:ln>
           <a:noFill/>
@@ -1430,6 +1430,310 @@
         </a:p>
       </xdr:txBody>
     </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>509654</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>33862</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>320179</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>77220</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="9" name="Picture 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C03F72A9-4CA6-4CA9-9AC5-AE5FF9719809}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
+          <a:lum bright="70000" contrast="-70000"/>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm rot="215940">
+          <a:off x="3578821" y="1557862"/>
+          <a:ext cx="424358" cy="424358"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>158752</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>31750</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>550334</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>42332</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="13" name="Picture 12">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8B544EAD-C94A-4B16-BB79-39A3A1337F9D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print">
+          <a:lum bright="70000" contrast="-70000"/>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5069419" y="1555750"/>
+          <a:ext cx="391582" cy="391582"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>381003</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>179917</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>179915</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>21163</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="15" name="Picture 14">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FE7E85CC-F32A-4450-8A60-B21CC9DDAEEA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3" cstate="print">
+          <a:lum bright="70000" contrast="-70000"/>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6519336" y="1513417"/>
+          <a:ext cx="412746" cy="412746"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>613832</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>7856</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>444500</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>71357</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="18" name="Picture 17">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BCADCC6E-6E43-4017-9CF3-4220FA3F07DE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4" cstate="print">
+          <a:lum bright="70000" contrast="-70000"/>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7979832" y="1531856"/>
+          <a:ext cx="444501" cy="444501"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>444501</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>190499</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>211669</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>1</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="20" name="Picture 19">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{58D534CD-904E-46C8-99B1-BA49E0377E33}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2899834" y="3047999"/>
+          <a:ext cx="381002" cy="381002"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>179918</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>74082</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>550334</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>63498</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="23" name="Picture 22">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AA7BBF00-41A2-450A-A8B1-5E7E9B9186E8}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8773585" y="3122082"/>
+          <a:ext cx="370416" cy="370416"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>

</xml_diff>